<commit_message>
fix: data type error in kode column in database.xlsx
</commit_message>
<xml_diff>
--- a/data/database.xlsx
+++ b/data/database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ridar\richard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2C8DF1-B815-49BD-A8F4-CAC296C742FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFB67A38-372E-475A-ACB5-4915D311922F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REALISASI" sheetId="2" r:id="rId1"/>
@@ -498,7 +498,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="69">
   <si>
     <t>Kode</t>
   </si>
@@ -509,58 +509,13 @@
     <t>FAKTOR PENGHAMBAT</t>
   </si>
   <si>
-    <t>5.01.01</t>
-  </si>
-  <si>
     <t>PPEPD</t>
-  </si>
-  <si>
-    <t>Penyusunan RKPD</t>
   </si>
   <si>
     <t>Dokumen</t>
   </si>
   <si>
-    <t>5.01.02</t>
-  </si>
-  <si>
-    <t>Musrenbang Kabupaten</t>
-  </si>
-  <si>
-    <t>Kali</t>
-  </si>
-  <si>
-    <t>5.02.01</t>
-  </si>
-  <si>
-    <t>Litbang</t>
-  </si>
-  <si>
-    <t>Kajian Strategis</t>
-  </si>
-  <si>
     <t>Laporan</t>
-  </si>
-  <si>
-    <t>5.03.01</t>
-  </si>
-  <si>
-    <t>Infrastruktur</t>
-  </si>
-  <si>
-    <t>Survey Lapangan</t>
-  </si>
-  <si>
-    <t>Titik</t>
-  </si>
-  <si>
-    <t>5.04.01</t>
-  </si>
-  <si>
-    <t>Pemerintahan</t>
-  </si>
-  <si>
-    <t>Penyusunan SOP</t>
   </si>
   <si>
     <t>Bidang</t>
@@ -602,21 +557,6 @@
     <t>Target Anggaran TW4</t>
   </si>
   <si>
-    <t>Proses pengadaan barang dan jasa mengalami keterlambatan sehingga pelaksanaan kegiatan belum dapat dimulai sesuai jadwal</t>
-  </si>
-  <si>
-    <t>Realisasi kegiatan terhambat karena kondisi cuaca yang tidak mendukung pelaksanaan pekerjaan di lapangan</t>
-  </si>
-  <si>
-    <t>Menyusun kembali jadwal pelaksanaan pekerjaan dengan mempertimbangkan prakiraan cuaca dan meningkatkan pengawasan terhadap progres pekerjaan</t>
-  </si>
-  <si>
-    <t>Keterbatasan jumlah tenaga pelaksana menyebabkan beberapa tahapan kegiatan belum dapat diselesaikan tepat waktu</t>
-  </si>
-  <si>
-    <t>Mengoptimalkan pembagian tugas serta melakukan penambahan personel atau dukungan tenaga teknis sesuai kebutuhan</t>
-  </si>
-  <si>
     <t>STATUS TINDAK LANJUT</t>
   </si>
   <si>
@@ -626,25 +566,145 @@
     <t>Catatan Tindak Lanjut</t>
   </si>
   <si>
-    <t>Percepat proses pengadaan dengan melakukan percepatan penyusunan dokumen dan koordinasi intensif dengan Unit Layanan Pengadaan (ULP)</t>
+    <t>PAGU</t>
   </si>
   <si>
-    <t>Selesai</t>
+    <t>REALISASI</t>
   </si>
   <si>
-    <t>Sementara Proses</t>
+    <t>Penyusunan dokumen perencanaan perangkat daerah</t>
   </si>
   <si>
-    <t>Belum Ditindaklanjuti</t>
+    <t xml:space="preserve">Evaluasi Kinerja Perangkat Daerah </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Penyediaan Gaji dan Tunjangan ASN </t>
+  </si>
+  <si>
+    <t>Sekretariat</t>
+  </si>
+  <si>
+    <t>Pelaksanaan Penatausahaan dan Pengujian/Verifikasi Keuangan SKPD</t>
+  </si>
+  <si>
+    <t>Pengamanan Barang Milik Daerah SKPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Penyediaan Peralatan dan Perlengkapan Kantor </t>
+  </si>
+  <si>
+    <t>Paket</t>
+  </si>
+  <si>
+    <t>Penyediaan Bahan Logistik Kantor</t>
+  </si>
+  <si>
+    <t>Penyediaan Barang Cetakan dan Penggandaan</t>
+  </si>
+  <si>
+    <t>Penyelenggaraan Rapat Koordinasi dan Konsultasi SKPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Penyediaan Jasa Komunikasi, Sumber Daya Air dan Listrik </t>
+  </si>
+  <si>
+    <t>Penyediaan Jasa Pemeliharaan, Biaya Pemeliharaan, Pajak, dan Perizinan Kendaraan Dinas Operasional atau Lapangan</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Pelaksanaan Musrenbang Kabupaten/Kota</t>
+  </si>
+  <si>
+    <t>Berita acara</t>
+  </si>
+  <si>
+    <t>Penyiapan Bahan Koordinasi Musrenbang Kecamatan</t>
+  </si>
+  <si>
+    <t>Usulan</t>
+  </si>
+  <si>
+    <t>Koordinasi Penyusunan dan Penetapan Dokumen Perencanaan Pembangunan Daerah Kabupaten/Kota</t>
+  </si>
+  <si>
+    <t>Koordinasi Pengendalian Perencanaan dan Pelaksanaan Pembangunan Daerah di Kabupaten/Kota</t>
+  </si>
+  <si>
+    <t>Monitoring, Evaluasi dan Penyusunan Laporan Berkala Pelaksanaan Pembangunan Daerah</t>
+  </si>
+  <si>
+    <t>Pengelolaan Data dalam Sistem Informasi Pemerintahan Daerah di Bidang Pembangunan Daerah</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Asistensi Penyusunan Dokumen Perencanaan Pembangunan Perangkat Daerah Bidang Pemerintahan</t>
+  </si>
+  <si>
+    <t>PPM</t>
+  </si>
+  <si>
+    <t>Koordinasi Pelaksanaan Sinergitas dan Harmonisasi Perencanaan Pembangunan Daerah Bidang Pemerintahan</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Asistensi Penyusunan Dokumen Perencanaan Pembangunan Perangkat Daerah Bidang Pembangunan Manusia</t>
+  </si>
+  <si>
+    <t>Koordinasi Pelaksanaan Sinergitas dan Harmonisasi Perencanaan Pembangunan Daerah Bidang Pembangunan Manusia</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Asistensi Penyusunan Dokumen Perencanaan Pembangunan Perangkat Daerah Bidang Perekonomian</t>
+  </si>
+  <si>
+    <t>Koordinasi Pelaksanaan Sinergitas dan Harmonisasi Perencanaan Pembangunan Daerah Bidang Perekonomian</t>
+  </si>
+  <si>
+    <t>Asistensi Penyusunan Dokumen Perencanaan Pembangunan Perangkat Daerah Bidang SDA</t>
+  </si>
+  <si>
+    <t>Koordinasi Pelaksanaan Sinergitas dan Harmonisasi Perencanaan Pembangunan Daerah Bidang SDA</t>
+  </si>
+  <si>
+    <t>PSDA</t>
+  </si>
+  <si>
+    <t>IK</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Asistensi Penyusunan Dokumen Perencanaan Pembangunan Perangkat Daerah Bidang Infrastruktur</t>
+  </si>
+  <si>
+    <t>Koordinasi Pelaksanaan Sinergitas dan Harmonisasi Perencanaan Pembangunan Daerah Bidang Infrastruktur</t>
+  </si>
+  <si>
+    <t>Asistensi Penyusunan Dokumen Perencanaan Pembangunan Perangkat Daerah Bidang Kewilayahan</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Koordinasi Pelaksanaan Sinergitas dan Harmonisasi Perencanaan Pembangunan Daerah Bidang Kewilayahan</t>
+  </si>
+  <si>
+    <t>RIDA</t>
+  </si>
+  <si>
+    <t>Penelitian dan Pengembangan Kesehatan</t>
+  </si>
+  <si>
+    <t>Uji Coba dan Penerapan Rancang Bangun/Model Replikasi dan Invensi di Bidang Difusi Inovasi dan Penerapan Teknologi</t>
+  </si>
+  <si>
+    <t>Penyusunan Rencana Aksi Pembangunan Kawasan Perbatasan</t>
+  </si>
+  <si>
+    <t>Administrasi pertanggung jawaban dari Kecamatan belum lengkap</t>
+  </si>
+  <si>
+    <t>Mdnghubungi pihak kecamatan untuk segera melengkapi pertanggung jawaban</t>
   </si>
   <si>
     <t>Diproses</t>
   </si>
   <si>
-    <t>PAGU</t>
-  </si>
-  <si>
-    <t>REALISASI</t>
+    <t>Sementara Proses</t>
   </si>
 </sst>
 </file>
@@ -723,7 +783,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -738,7 +798,27 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Comma [0] 12" xfId="7" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -1417,6 +1497,9 @@
 <file path=xl/externalLinks/externalLink14.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Master Penjabarn APBD"/>
       <sheetName val="master utk setda"/>
@@ -1701,6 +1784,9 @@
 <file path=xl/externalLinks/externalLink16.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Master Penjabarn APBD"/>
       <sheetName val="master utk setda"/>
@@ -1864,6 +1950,9 @@
 <file path=xl/externalLinks/externalLink17.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Master Penjabarn APBD"/>
       <sheetName val="master utk setda"/>
@@ -1985,6 +2074,9 @@
 <file path=xl/externalLinks/externalLink18.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Master Penjabarn APBD"/>
       <sheetName val="master utk setda"/>
@@ -2799,6 +2891,9 @@
 <file path=xl/externalLinks/externalLink23.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Master Penjabarn APBD"/>
       <sheetName val="master utk setda"/>
@@ -11193,6 +11288,9 @@
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Master Penjabarn APBD"/>
       <sheetName val="master utk setda"/>
@@ -11664,6 +11762,9 @@
 <file path=xl/externalLinks/externalLink7.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Master Penjabarn APBD"/>
       <sheetName val="master utk setda"/>
@@ -12248,57 +12349,57 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CC386AA-95CB-4959-8185-395B0BDC2271}">
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.08984375" customWidth="1"/>
+    <col min="2" max="2" width="12.08984375" customWidth="1"/>
+    <col min="3" max="3" width="31.36328125" customWidth="1"/>
     <col min="4" max="4" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.90625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.36328125" bestFit="1" customWidth="1"/>
     <col min="7" max="10" width="20.7265625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="20.7265625" customWidth="1"/>
-    <col min="12" max="12" width="20" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="25.26953125" customWidth="1"/>
+    <col min="13" max="13" width="23.1796875" customWidth="1"/>
     <col min="14" max="14" width="20.7265625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="19.1796875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="19.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>48</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>2</v>
@@ -12307,39 +12408,39 @@
         <v>1</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
+      <c r="A2" s="2">
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="2">
+        <v>12</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="2">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>6</v>
-      </c>
       <c r="F2" s="2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G2" s="3">
-        <v>25000000</v>
+        <v>1099500</v>
       </c>
       <c r="H2" s="3">
-        <v>30000000</v>
+        <v>682500</v>
       </c>
       <c r="I2" s="2">
         <v>0</v>
@@ -12349,36 +12450,36 @@
       </c>
       <c r="K2" s="3">
         <f>SUM(G2:J2)</f>
-        <v>55000000</v>
+        <v>1782000</v>
       </c>
       <c r="L2" s="4"/>
       <c r="M2" s="4"/>
       <c r="O2" s="5"/>
     </row>
-    <row r="3" spans="1:16" ht="217.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="2">
         <v>7</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="2">
-        <v>10</v>
-      </c>
       <c r="E3" s="2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F3" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G3" s="3">
-        <v>15000000</v>
+        <v>1171000</v>
       </c>
       <c r="H3" s="3">
-        <v>20000000</v>
+        <v>682500</v>
       </c>
       <c r="I3" s="2">
         <v>0</v>
@@ -12387,44 +12488,37 @@
         <v>0</v>
       </c>
       <c r="K3" s="3">
-        <f t="shared" ref="K3:K6" si="0">SUM(G3:J3)</f>
-        <v>35000000</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="N3" t="s">
-        <v>45</v>
-      </c>
+        <f t="shared" ref="K3:K9" si="0">SUM(G3:J3)</f>
+        <v>1853500</v>
+      </c>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
       <c r="O3" s="5"/>
     </row>
-    <row r="4" spans="1:16" ht="145" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="D4" s="2">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="F4" s="2">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="G4" s="3">
-        <v>10000000</v>
+        <v>700345518</v>
       </c>
       <c r="H4" s="3">
-        <v>15000000</v>
+        <v>707220957</v>
       </c>
       <c r="I4" s="2">
         <v>0</v>
@@ -12434,46 +12528,36 @@
       </c>
       <c r="K4" s="3">
         <f t="shared" si="0"/>
-        <v>25000000</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="N4" t="s">
-        <v>46</v>
-      </c>
+        <v>1407566475</v>
+      </c>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
       <c r="O4" s="5"/>
-      <c r="P4" t="s">
-        <v>44</v>
-      </c>
     </row>
-    <row r="5" spans="1:16" ht="203" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>14</v>
+    <row r="5" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="D5" s="2">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="F5" s="2">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3">
-        <v>5000000</v>
+        <v>403000</v>
       </c>
       <c r="H5" s="3">
-        <v>10000000</v>
+        <v>12103000</v>
       </c>
       <c r="I5" s="2">
         <v>0</v>
@@ -12483,45 +12567,37 @@
       </c>
       <c r="K5" s="3">
         <f t="shared" si="0"/>
-        <v>15000000</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="N5" t="s">
-        <v>43</v>
-      </c>
-      <c r="O5" s="5">
-        <v>53160</v>
-      </c>
+        <v>12506000</v>
+      </c>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="5"/>
     </row>
-    <row r="6" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>18</v>
+    <row r="6" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D6" s="2">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F6" s="2">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G6" s="3">
-        <v>40000000</v>
+        <v>100000</v>
       </c>
       <c r="H6" s="3">
-        <v>35000000</v>
+        <v>850000</v>
       </c>
       <c r="I6" s="2">
         <v>0</v>
@@ -12531,11 +12607,995 @@
       </c>
       <c r="K6" s="3">
         <f t="shared" si="0"/>
-        <v>75000000</v>
+        <v>950000</v>
       </c>
       <c r="L6" s="4"/>
       <c r="M6" s="4"/>
       <c r="O6" s="5"/>
+    </row>
+    <row r="7" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="2">
+        <v>11</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="2">
+        <v>11</v>
+      </c>
+      <c r="G7" s="3">
+        <v>8109000</v>
+      </c>
+      <c r="H7" s="3">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0</v>
+      </c>
+      <c r="K7" s="3">
+        <f t="shared" si="0"/>
+        <v>8109000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="2">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="3">
+        <v>1</v>
+      </c>
+      <c r="G8" s="3">
+        <v>4121500</v>
+      </c>
+      <c r="H8" s="6">
+        <v>4121500</v>
+      </c>
+      <c r="I8" s="3">
+        <v>0</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0</v>
+      </c>
+      <c r="K8" s="3">
+        <f t="shared" si="0"/>
+        <v>8243000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="2">
+        <v>2</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" s="3">
+        <v>2</v>
+      </c>
+      <c r="G9" s="3">
+        <v>1500000</v>
+      </c>
+      <c r="H9" s="3">
+        <v>1228000</v>
+      </c>
+      <c r="I9" s="3">
+        <v>0</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3">
+        <f t="shared" si="0"/>
+        <v>2728000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="2">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0</v>
+      </c>
+      <c r="H10" s="3">
+        <v>7580700</v>
+      </c>
+      <c r="I10" s="3">
+        <v>0</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0</v>
+      </c>
+      <c r="K10" s="3">
+        <f t="shared" ref="K10:K18" si="1">SUM(G10:J10)</f>
+        <v>7580700</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="2">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F11" s="3">
+        <v>0</v>
+      </c>
+      <c r="G11" s="3">
+        <v>18339800</v>
+      </c>
+      <c r="H11" s="3">
+        <v>40019700</v>
+      </c>
+      <c r="I11" s="3">
+        <v>0</v>
+      </c>
+      <c r="J11" s="2">
+        <v>0</v>
+      </c>
+      <c r="K11" s="3">
+        <f t="shared" si="1"/>
+        <v>58359500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="2">
+        <v>14</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" s="3">
+        <v>0</v>
+      </c>
+      <c r="G12" s="3">
+        <v>1995000</v>
+      </c>
+      <c r="H12" s="3">
+        <v>13178400</v>
+      </c>
+      <c r="I12" s="3">
+        <v>0</v>
+      </c>
+      <c r="J12" s="2">
+        <v>0</v>
+      </c>
+      <c r="K12" s="3">
+        <f t="shared" si="1"/>
+        <v>15173400</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="2">
+        <v>2</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F13" s="3">
+        <v>2</v>
+      </c>
+      <c r="G13" s="3">
+        <v>655000</v>
+      </c>
+      <c r="H13" s="3">
+        <v>13249000</v>
+      </c>
+      <c r="I13" s="3">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0</v>
+      </c>
+      <c r="K13" s="3">
+        <f t="shared" si="1"/>
+        <v>13904000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="2">
+        <v>11</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F14" s="3">
+        <v>11</v>
+      </c>
+      <c r="G14" s="3">
+        <v>9342500</v>
+      </c>
+      <c r="H14" s="3">
+        <v>56767500</v>
+      </c>
+      <c r="I14" s="3">
+        <v>0</v>
+      </c>
+      <c r="J14" s="2">
+        <v>0</v>
+      </c>
+      <c r="K14" s="3">
+        <f t="shared" si="1"/>
+        <v>66110000</v>
+      </c>
+      <c r="L14" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="M14" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="N14" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="P14" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="2">
+        <v>2</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F15" s="3">
+        <v>1</v>
+      </c>
+      <c r="G15" s="3">
+        <v>2695000</v>
+      </c>
+      <c r="H15" s="3">
+        <v>15533500</v>
+      </c>
+      <c r="I15" s="3">
+        <v>0</v>
+      </c>
+      <c r="J15" s="2">
+        <v>0</v>
+      </c>
+      <c r="K15" s="3">
+        <f t="shared" si="1"/>
+        <v>18228500</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D16" s="2">
+        <v>4</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F16" s="3">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3">
+        <v>130000</v>
+      </c>
+      <c r="H16" s="3">
+        <v>223000</v>
+      </c>
+      <c r="I16" s="3">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2">
+        <v>0</v>
+      </c>
+      <c r="K16" s="3">
+        <f t="shared" si="1"/>
+        <v>353000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="2">
+        <v>4</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F17" s="3">
+        <v>1</v>
+      </c>
+      <c r="G17" s="3">
+        <v>400000</v>
+      </c>
+      <c r="H17" s="3">
+        <v>10147400</v>
+      </c>
+      <c r="I17" s="3">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2">
+        <v>0</v>
+      </c>
+      <c r="K17" s="3">
+        <f t="shared" si="1"/>
+        <v>10547400</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="2">
+        <v>1</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F18" s="3">
+        <v>0</v>
+      </c>
+      <c r="G18" s="3">
+        <v>815000</v>
+      </c>
+      <c r="H18" s="3">
+        <v>5780000</v>
+      </c>
+      <c r="I18" s="3">
+        <v>0</v>
+      </c>
+      <c r="J18" s="2">
+        <v>0</v>
+      </c>
+      <c r="K18" s="3">
+        <f t="shared" si="1"/>
+        <v>6595000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="2">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F19" s="3">
+        <v>0</v>
+      </c>
+      <c r="G19" s="3">
+        <v>4201600</v>
+      </c>
+      <c r="H19" s="3">
+        <v>4547000</v>
+      </c>
+      <c r="I19" s="3">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2">
+        <v>0</v>
+      </c>
+      <c r="K19" s="3">
+        <f t="shared" ref="K19:K33" si="2">SUM(G19:J19)</f>
+        <v>8748600</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="2">
+        <v>1</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F20" s="3">
+        <v>0</v>
+      </c>
+      <c r="G20" s="3">
+        <v>3137400</v>
+      </c>
+      <c r="H20" s="3">
+        <v>3125500</v>
+      </c>
+      <c r="I20" s="3">
+        <v>0</v>
+      </c>
+      <c r="J20" s="2">
+        <v>0</v>
+      </c>
+      <c r="K20" s="3">
+        <f t="shared" si="2"/>
+        <v>6262900</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" s="2">
+        <v>1</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F21" s="3">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3">
+        <v>154800</v>
+      </c>
+      <c r="H21" s="3">
+        <v>3360000</v>
+      </c>
+      <c r="I21" s="3">
+        <v>0</v>
+      </c>
+      <c r="J21" s="2">
+        <v>0</v>
+      </c>
+      <c r="K21" s="3">
+        <f t="shared" si="2"/>
+        <v>3514800</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D22" s="2">
+        <v>1</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F22" s="3">
+        <v>0</v>
+      </c>
+      <c r="G22" s="3">
+        <v>4373000</v>
+      </c>
+      <c r="H22" s="3">
+        <v>4185000</v>
+      </c>
+      <c r="I22" s="3">
+        <v>0</v>
+      </c>
+      <c r="J22" s="2">
+        <v>0</v>
+      </c>
+      <c r="K22" s="3">
+        <f t="shared" si="2"/>
+        <v>8558000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A23" s="2">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" s="2">
+        <v>1</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F23" s="3">
+        <v>0</v>
+      </c>
+      <c r="G23" s="3">
+        <v>5104800</v>
+      </c>
+      <c r="H23" s="3">
+        <v>0</v>
+      </c>
+      <c r="I23" s="3">
+        <v>0</v>
+      </c>
+      <c r="J23" s="2">
+        <v>0</v>
+      </c>
+      <c r="K23" s="3">
+        <f t="shared" si="2"/>
+        <v>5104800</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D24" s="2">
+        <v>1</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F24" s="3">
+        <v>0</v>
+      </c>
+      <c r="G24" s="3">
+        <v>1766000</v>
+      </c>
+      <c r="H24" s="3">
+        <v>4959000</v>
+      </c>
+      <c r="I24" s="3">
+        <v>0</v>
+      </c>
+      <c r="J24" s="2">
+        <v>0</v>
+      </c>
+      <c r="K24" s="3">
+        <f t="shared" si="2"/>
+        <v>6725000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D25" s="2">
+        <v>1</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F25" s="3">
+        <v>0</v>
+      </c>
+      <c r="G25" s="3">
+        <v>3221700</v>
+      </c>
+      <c r="H25" s="3">
+        <v>113500</v>
+      </c>
+      <c r="I25" s="3">
+        <v>0</v>
+      </c>
+      <c r="J25" s="2">
+        <v>0</v>
+      </c>
+      <c r="K25" s="3">
+        <f t="shared" si="2"/>
+        <v>3335200</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D26" s="2">
+        <v>1</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F26" s="3">
+        <v>0</v>
+      </c>
+      <c r="G26" s="3">
+        <v>4678800</v>
+      </c>
+      <c r="H26" s="3">
+        <v>8687000</v>
+      </c>
+      <c r="I26" s="3">
+        <v>0</v>
+      </c>
+      <c r="J26" s="2">
+        <v>0</v>
+      </c>
+      <c r="K26" s="3">
+        <f t="shared" si="2"/>
+        <v>13365800</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D27" s="2">
+        <v>1</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F27" s="3">
+        <v>0</v>
+      </c>
+      <c r="G27" s="3">
+        <v>2569600</v>
+      </c>
+      <c r="H27" s="3">
+        <v>728500</v>
+      </c>
+      <c r="I27" s="3">
+        <v>0</v>
+      </c>
+      <c r="J27" s="2">
+        <v>0</v>
+      </c>
+      <c r="K27" s="3">
+        <f t="shared" si="2"/>
+        <v>3298100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D28" s="2">
+        <v>1</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F28" s="3">
+        <v>0</v>
+      </c>
+      <c r="G28" s="3">
+        <v>3985000</v>
+      </c>
+      <c r="H28" s="3">
+        <v>3481900</v>
+      </c>
+      <c r="I28" s="3">
+        <v>0</v>
+      </c>
+      <c r="J28" s="2">
+        <v>0</v>
+      </c>
+      <c r="K28" s="3">
+        <f t="shared" si="2"/>
+        <v>7466900</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D29" s="2">
+        <v>1</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F29" s="3">
+        <v>0</v>
+      </c>
+      <c r="G29" s="3">
+        <v>1797000</v>
+      </c>
+      <c r="H29" s="3">
+        <v>0</v>
+      </c>
+      <c r="I29" s="3">
+        <v>0</v>
+      </c>
+      <c r="J29" s="2">
+        <v>0</v>
+      </c>
+      <c r="K29" s="3">
+        <f t="shared" si="2"/>
+        <v>1797000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D30" s="2">
+        <v>1</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F30" s="3">
+        <v>0</v>
+      </c>
+      <c r="G30" s="3">
+        <v>1700000</v>
+      </c>
+      <c r="H30" s="3">
+        <v>5738000</v>
+      </c>
+      <c r="I30" s="3">
+        <v>0</v>
+      </c>
+      <c r="J30" s="3">
+        <v>0</v>
+      </c>
+      <c r="K30" s="3">
+        <f t="shared" si="2"/>
+        <v>7438000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A31" s="2">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D31" s="2">
+        <v>1</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F31" s="3">
+        <v>0</v>
+      </c>
+      <c r="G31" s="3">
+        <v>1605000</v>
+      </c>
+      <c r="H31" s="3">
+        <v>8437300</v>
+      </c>
+      <c r="I31" s="3">
+        <v>0</v>
+      </c>
+      <c r="J31" s="2">
+        <v>0</v>
+      </c>
+      <c r="K31" s="3">
+        <f t="shared" si="2"/>
+        <v>10042300</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A32" s="2">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D32" s="2">
+        <v>5</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F32" s="3">
+        <v>0</v>
+      </c>
+      <c r="G32" s="3">
+        <v>2938000</v>
+      </c>
+      <c r="H32" s="3">
+        <v>24260000</v>
+      </c>
+      <c r="I32" s="3">
+        <v>0</v>
+      </c>
+      <c r="J32" s="2">
+        <v>0</v>
+      </c>
+      <c r="K32" s="3">
+        <f t="shared" si="2"/>
+        <v>27198000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A33" s="2">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D33" s="2">
+        <v>1</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F33" s="3">
+        <v>0</v>
+      </c>
+      <c r="G33" s="3">
+        <v>0</v>
+      </c>
+      <c r="H33" s="3">
+        <v>3555900</v>
+      </c>
+      <c r="I33" s="3">
+        <v>0</v>
+      </c>
+      <c r="J33" s="2">
+        <v>0</v>
+      </c>
+      <c r="K33" s="3">
+        <f t="shared" si="2"/>
+        <v>3555900</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -12545,14 +13605,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB74AF2A-0A41-4E24-8264-D3815A13712E}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" customWidth="1"/>
+    <col min="3" max="3" width="30.7265625" customWidth="1"/>
     <col min="4" max="7" width="19" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
@@ -12560,160 +13620,889 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
+      <c r="A2" s="2">
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="D2" s="3">
-        <v>30000000</v>
+        <v>1099500</v>
       </c>
       <c r="E2" s="3">
-        <v>35000000</v>
+        <v>682500</v>
       </c>
       <c r="F2" s="3">
-        <v>20000000</v>
+        <v>0</v>
       </c>
       <c r="G2" s="3">
-        <v>15000000</v>
-      </c>
-      <c r="H2" s="6">
+        <v>0</v>
+      </c>
+      <c r="H2" s="8">
         <f>SUM(D2:G2)</f>
-        <v>100000000</v>
+        <v>1782000</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>7</v>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="D3" s="3">
-        <v>20000000</v>
+        <v>1171000</v>
       </c>
       <c r="E3" s="3">
-        <v>25000000</v>
+        <v>682500</v>
       </c>
       <c r="F3" s="3">
-        <v>20000000</v>
+        <v>0</v>
       </c>
       <c r="G3" s="3">
-        <v>15000000</v>
-      </c>
-      <c r="H3" s="6">
-        <f t="shared" ref="H3:H6" si="0">SUM(D3:G3)</f>
-        <v>80000000</v>
+        <v>0</v>
+      </c>
+      <c r="H3" s="8">
+        <f t="shared" ref="H3:H33" si="0">SUM(D3:G3)</f>
+        <v>1853500</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="3">
+        <v>796747205</v>
+      </c>
+      <c r="E4" s="3">
+        <v>732460327</v>
+      </c>
+      <c r="F4" s="3">
+        <v>740266285</v>
+      </c>
+      <c r="G4" s="3">
+        <v>513502599</v>
+      </c>
+      <c r="H4" s="8">
+        <f t="shared" si="0"/>
+        <v>2782976416</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="3">
+        <v>403000</v>
+      </c>
+      <c r="E5" s="3">
+        <v>11700000</v>
+      </c>
+      <c r="F5" s="3">
+        <v>23400000</v>
+      </c>
+      <c r="G5" s="3">
+        <v>11700000</v>
+      </c>
+      <c r="H5" s="8">
+        <f t="shared" si="0"/>
+        <v>47203000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="3">
+        <v>850000</v>
+      </c>
+      <c r="E6" s="3">
+        <v>750000</v>
+      </c>
+      <c r="F6" s="3">
+        <v>750000</v>
+      </c>
+      <c r="G6" s="3">
+        <v>750000</v>
+      </c>
+      <c r="H6" s="8">
+        <f t="shared" si="0"/>
+        <v>3100000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="3">
+        <v>7659000</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3">
+        <v>450000</v>
+      </c>
+      <c r="H7" s="8">
+        <f t="shared" si="0"/>
+        <v>8109000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="3">
+        <v>4121500</v>
+      </c>
+      <c r="E8" s="3">
+        <v>4121500</v>
+      </c>
+      <c r="F8" s="3">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3">
+        <v>0</v>
+      </c>
+      <c r="H8" s="8">
+        <f t="shared" si="0"/>
+        <v>8243000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1500000</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1228000</v>
+      </c>
+      <c r="F9" s="3">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3">
+        <v>0</v>
+      </c>
+      <c r="H9" s="8">
+        <f t="shared" si="0"/>
+        <v>2728000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="3">
+        <v>10590700</v>
+      </c>
+      <c r="E10" s="3">
+        <v>12365300</v>
+      </c>
+      <c r="F10" s="3">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3">
+        <v>0</v>
+      </c>
+      <c r="H10" s="8">
+        <f t="shared" si="0"/>
+        <v>22956000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="3">
+        <v>26100000</v>
+      </c>
+      <c r="E11" s="3">
+        <v>19200000</v>
+      </c>
+      <c r="F11" s="3">
+        <v>19200000</v>
+      </c>
+      <c r="G11" s="3">
+        <v>18668000</v>
+      </c>
+      <c r="H11" s="8">
+        <f t="shared" si="0"/>
+        <v>83168000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="B12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="3">
+        <v>7774000</v>
+      </c>
+      <c r="E12" s="3">
+        <v>7500000</v>
+      </c>
+      <c r="F12" s="3">
+        <v>7601300</v>
+      </c>
+      <c r="G12" s="3">
+        <v>6935000</v>
+      </c>
+      <c r="H12" s="8">
+        <f t="shared" si="0"/>
+        <v>29810300</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="2">
         <v>12</v>
       </c>
-      <c r="D4" s="3">
-        <v>15000000</v>
-      </c>
-      <c r="E4" s="3">
-        <v>20000000</v>
-      </c>
-      <c r="F4" s="3">
-        <v>10000000</v>
-      </c>
-      <c r="G4" s="3">
-        <v>5000000</v>
-      </c>
-      <c r="H4" s="6">
+      <c r="B13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="3">
+        <v>855000</v>
+      </c>
+      <c r="E13" s="3">
+        <v>16854000</v>
+      </c>
+      <c r="F13" s="3">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3">
+        <v>5600000</v>
+      </c>
+      <c r="H13" s="8">
         <f t="shared" si="0"/>
-        <v>50000000</v>
+        <v>23309000</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+    <row r="14" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="3">
+        <v>9409500</v>
+      </c>
+      <c r="E14" s="3">
+        <v>109000000</v>
+      </c>
+      <c r="F14" s="3">
+        <v>0</v>
+      </c>
+      <c r="G14" s="3">
+        <v>0</v>
+      </c>
+      <c r="H14" s="8">
+        <f t="shared" si="0"/>
+        <v>118409500</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A15" s="2">
         <v>14</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="3">
+        <v>7920500</v>
+      </c>
+      <c r="E15" s="3">
+        <v>27437500</v>
+      </c>
+      <c r="F15" s="3">
+        <v>2506000</v>
+      </c>
+      <c r="G15" s="3">
+        <v>2700000</v>
+      </c>
+      <c r="H15" s="8">
+        <f t="shared" si="0"/>
+        <v>40564000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A16" s="2">
         <v>15</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="B16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D16" s="3">
+        <v>130000</v>
+      </c>
+      <c r="E16" s="3">
+        <v>3447500</v>
+      </c>
+      <c r="F16" s="3">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3">
+        <v>3419000</v>
+      </c>
+      <c r="H16" s="8">
+        <f t="shared" si="0"/>
+        <v>6996500</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="2">
         <v>16</v>
       </c>
-      <c r="D5" s="3">
-        <v>10000000</v>
-      </c>
-      <c r="E5" s="3">
-        <v>15000000</v>
-      </c>
-      <c r="F5" s="3">
-        <v>10000000</v>
-      </c>
-      <c r="G5" s="3">
-        <v>5000000</v>
-      </c>
-      <c r="H5" s="6">
+      <c r="B17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="3">
+        <v>2005400</v>
+      </c>
+      <c r="E17" s="3">
+        <v>8152000</v>
+      </c>
+      <c r="F17" s="3">
+        <v>9653400</v>
+      </c>
+      <c r="G17" s="3">
+        <v>0</v>
+      </c>
+      <c r="H17" s="8">
         <f t="shared" si="0"/>
-        <v>40000000</v>
+        <v>19810800</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+    <row r="18" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="3">
+        <v>815000</v>
+      </c>
+      <c r="E18" s="3">
+        <v>8252000</v>
+      </c>
+      <c r="F18" s="3">
+        <v>965800</v>
+      </c>
+      <c r="G18" s="3">
+        <v>0</v>
+      </c>
+      <c r="H18" s="8">
+        <f t="shared" si="0"/>
+        <v>10032800</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A19" s="2">
         <v>18</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B19" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="3">
+        <v>7466600</v>
+      </c>
+      <c r="E19" s="3">
+        <v>3732000</v>
+      </c>
+      <c r="F19" s="3">
+        <v>0</v>
+      </c>
+      <c r="G19" s="3">
+        <v>0</v>
+      </c>
+      <c r="H19" s="8">
+        <f t="shared" si="0"/>
+        <v>11198600</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A20" s="2">
         <v>19</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="B20" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="3">
+        <v>3137400</v>
+      </c>
+      <c r="E20" s="3">
+        <v>4339000</v>
+      </c>
+      <c r="F20" s="3">
+        <v>6000000</v>
+      </c>
+      <c r="G20" s="3">
+        <v>4000000</v>
+      </c>
+      <c r="H20" s="8">
+        <f t="shared" si="0"/>
+        <v>17476400</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A21" s="2">
         <v>20</v>
       </c>
-      <c r="D6" s="3">
-        <v>35000000</v>
-      </c>
-      <c r="E6" s="3">
-        <v>35000000</v>
-      </c>
-      <c r="F6" s="3">
-        <v>20000000</v>
-      </c>
-      <c r="G6" s="3">
-        <v>10000000</v>
-      </c>
-      <c r="H6" s="6">
+      <c r="B21" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" s="3">
+        <v>3514800</v>
+      </c>
+      <c r="E21" s="3">
+        <v>2720000</v>
+      </c>
+      <c r="F21" s="3">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3">
+        <v>0</v>
+      </c>
+      <c r="H21" s="8">
         <f t="shared" si="0"/>
-        <v>100000000</v>
+        <v>6234800</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D22" s="3">
+        <v>8226000</v>
+      </c>
+      <c r="E22" s="3">
+        <v>381000</v>
+      </c>
+      <c r="F22" s="3">
+        <v>10160000</v>
+      </c>
+      <c r="G22" s="3">
+        <v>0</v>
+      </c>
+      <c r="H22" s="8">
+        <f t="shared" si="0"/>
+        <v>18767000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A23" s="2">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" s="3">
+        <v>5104800</v>
+      </c>
+      <c r="E23" s="3">
+        <v>0</v>
+      </c>
+      <c r="F23" s="3">
+        <v>0</v>
+      </c>
+      <c r="G23" s="3">
+        <v>0</v>
+      </c>
+      <c r="H23" s="8">
+        <f t="shared" si="0"/>
+        <v>5104800</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D24" s="3">
+        <v>2616000</v>
+      </c>
+      <c r="E24" s="3">
+        <v>4109000</v>
+      </c>
+      <c r="F24" s="3">
+        <v>71469500</v>
+      </c>
+      <c r="G24" s="3">
+        <v>0</v>
+      </c>
+      <c r="H24" s="8">
+        <f t="shared" si="0"/>
+        <v>78194500</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D25" s="3">
+        <v>3221700</v>
+      </c>
+      <c r="E25" s="3">
+        <v>2056500</v>
+      </c>
+      <c r="F25" s="3">
+        <v>0</v>
+      </c>
+      <c r="G25" s="3">
+        <v>0</v>
+      </c>
+      <c r="H25" s="8">
+        <f t="shared" si="0"/>
+        <v>5278200</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D26" s="3">
+        <v>5678800</v>
+      </c>
+      <c r="E26" s="3">
+        <v>8077000</v>
+      </c>
+      <c r="F26" s="3">
+        <v>357000</v>
+      </c>
+      <c r="G26" s="3">
+        <v>0</v>
+      </c>
+      <c r="H26" s="8">
+        <f t="shared" si="0"/>
+        <v>14112800</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D27" s="3">
+        <v>2569600</v>
+      </c>
+      <c r="E27" s="3">
+        <v>728500</v>
+      </c>
+      <c r="F27" s="3">
+        <v>844600</v>
+      </c>
+      <c r="G27" s="3">
+        <v>757000</v>
+      </c>
+      <c r="H27" s="8">
+        <f t="shared" si="0"/>
+        <v>4899700</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="D28" s="3">
+        <v>7811000</v>
+      </c>
+      <c r="E28" s="3">
+        <v>100000</v>
+      </c>
+      <c r="F28" s="3">
+        <v>2506000</v>
+      </c>
+      <c r="G28" s="3">
+        <v>131200</v>
+      </c>
+      <c r="H28" s="8">
+        <f t="shared" si="0"/>
+        <v>10548200</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D29" s="3">
+        <v>1797000</v>
+      </c>
+      <c r="E29" s="3">
+        <v>1107000</v>
+      </c>
+      <c r="F29" s="3">
+        <v>1107000</v>
+      </c>
+      <c r="G29" s="3">
+        <v>1213000</v>
+      </c>
+      <c r="H29" s="8">
+        <f t="shared" si="0"/>
+        <v>5224000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D30" s="3">
+        <v>1700000</v>
+      </c>
+      <c r="E30" s="3">
+        <v>18499000</v>
+      </c>
+      <c r="F30" s="3">
+        <v>2484000</v>
+      </c>
+      <c r="G30" s="3">
+        <v>131600</v>
+      </c>
+      <c r="H30" s="8">
+        <f t="shared" si="0"/>
+        <v>22814600</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A31" s="2">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D31" s="3">
+        <v>3285600</v>
+      </c>
+      <c r="E31" s="3">
+        <v>42166500</v>
+      </c>
+      <c r="F31" s="3">
+        <v>23250000</v>
+      </c>
+      <c r="G31" s="3">
+        <v>0</v>
+      </c>
+      <c r="H31" s="8">
+        <f t="shared" si="0"/>
+        <v>68702100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A32" s="2">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D32" s="3">
+        <v>3088100</v>
+      </c>
+      <c r="E32" s="3">
+        <v>43901750</v>
+      </c>
+      <c r="F32" s="3">
+        <v>28569750</v>
+      </c>
+      <c r="G32" s="3">
+        <v>18100000</v>
+      </c>
+      <c r="H32" s="8">
+        <f t="shared" si="0"/>
+        <v>93659600</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="2">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D33" s="3">
+        <v>0</v>
+      </c>
+      <c r="E33" s="3">
+        <v>3826000</v>
+      </c>
+      <c r="F33" s="3">
+        <v>957100</v>
+      </c>
+      <c r="G33" s="3">
+        <v>655500</v>
+      </c>
+      <c r="H33" s="8">
+        <f t="shared" si="0"/>
+        <v>5438600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>